<commit_message>
Add a workshop category, and a way to get new list values into a workbook
One category for the workshop end of the lab: 3D printers, pillar drills, saws,
grinders, soldering stations. Hand tools and clamps stay items, on the items
sheet, where the tool category now says so. TOOL joins the suggested id
prefixes, and the drawing has a colour for it.

A category in the blank template is no use in a workbook made before it existed:
the value isn't in that file's lists sheet, so Excel's dropdown refuses it and
the checks report it as not on the list. `python -m labmap lists` copies over
whatever the template has gained, stretches each dropdown's named range across
the new rows, and leaves values of its own alone, writing cell by cell so the
rest of the workbook is untouched.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/example/lab-data.original.xlsx
+++ b/example/lab-data.original.xlsx
@@ -21,7 +21,7 @@
     <sheet name="lists" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
-    <definedName name="L_category">lists!$A$2:$A$44</definedName>
+    <definedName name="L_category">lists!$A$2:$A$45</definedName>
     <definedName name="L_mount">lists!$D$2:$D$7</definedName>
     <definedName name="L_faces">lists!$G$2:$G$9</definedName>
     <definedName name="L_shape">lists!$J$2:$J$5</definedName>
@@ -1996,7 +1996,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BG57"/>
+  <dimension ref="A1:BG58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2383,6 +2383,11 @@
           <t>tool</t>
         </is>
       </c>
+      <c r="AO2" t="inlineStr">
+        <is>
+          <t>hand tools: clamps, saws, drivers, files</t>
+        </is>
+      </c>
       <c r="AQ2" t="inlineStr">
         <is>
           <t>none</t>
@@ -3780,12 +3785,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>computer</t>
+          <t>workshop</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>PC, controller</t>
+          <t>workshop machine or tool: 3D printer, drill, saw, grinder, soldering station</t>
         </is>
       </c>
       <c r="BF31" t="inlineStr">
@@ -3802,12 +3807,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>monitor</t>
+          <t>computer</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>screen</t>
+          <t>PC, controller</t>
         </is>
       </c>
       <c r="BF32" t="inlineStr">
@@ -3824,12 +3829,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ups</t>
+          <t>monitor</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>uninterruptible power supply</t>
+          <t>screen</t>
         </is>
       </c>
       <c r="BF33" t="inlineStr">
@@ -3846,12 +3851,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>fridge</t>
+          <t>ups</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>fridge: solvents, inks, samples</t>
+          <t>uninterruptible power supply</t>
         </is>
       </c>
       <c r="BF34" t="inlineStr">
@@ -3868,369 +3873,391 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>freezer</t>
+          <t>fridge</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>freezer: precursors, samples</t>
+          <t>fridge: solvents, inks, samples</t>
         </is>
       </c>
       <c r="BF35" t="inlineStr">
         <is>
-          <t>PC</t>
+          <t>TOOL</t>
         </is>
       </c>
       <c r="BG35" t="inlineStr">
         <is>
-          <t>computer</t>
+          <t>workshop machine or tool</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>gas-cylinder</t>
+          <t>freezer</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>gas cylinder</t>
+          <t>freezer: precursors, samples</t>
         </is>
       </c>
       <c r="BF36" t="inlineStr">
         <is>
-          <t>MON</t>
+          <t>PC</t>
         </is>
       </c>
       <c r="BG36" t="inlineStr">
         <is>
-          <t>monitor</t>
+          <t>computer</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>sink</t>
+          <t>gas-cylinder</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>sink bowl, drainer</t>
+          <t>gas cylinder</t>
         </is>
       </c>
       <c r="BF37" t="inlineStr">
         <is>
-          <t>UPS</t>
+          <t>MON</t>
         </is>
       </c>
       <c r="BG37" t="inlineStr">
         <is>
-          <t>UPS</t>
+          <t>monitor</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>safety</t>
+          <t>sink</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>eyewash, shower, extinguisher, spill kit, emergency stop</t>
+          <t>sink bowl, drainer</t>
         </is>
       </c>
       <c r="BF38" t="inlineStr">
         <is>
-          <t>FRG</t>
+          <t>UPS</t>
         </is>
       </c>
       <c r="BG38" t="inlineStr">
         <is>
-          <t>fridge</t>
+          <t>UPS</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>structure</t>
+          <t>safety</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>column, pipe boxing, radiator, electrical panel</t>
+          <t>eyewash, shower, extinguisher, spill kit, emergency stop</t>
         </is>
       </c>
       <c r="BF39" t="inlineStr">
         <is>
-          <t>FRZ</t>
+          <t>FRG</t>
         </is>
       </c>
       <c r="BG39" t="inlineStr">
         <is>
-          <t>freezer</t>
+          <t>fridge</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>door</t>
+          <t>structure</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>door; clear_front = swing</t>
+          <t>column, pipe boxing, radiator, electrical panel</t>
         </is>
       </c>
       <c r="BF40" t="inlineStr">
         <is>
-          <t>GAS</t>
+          <t>FRZ</t>
         </is>
       </c>
       <c r="BG40" t="inlineStr">
         <is>
-          <t>gas cylinder</t>
+          <t>freezer</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>window</t>
+          <t>door</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>mount = wall, z = sill height</t>
+          <t>door; clear_front = swing</t>
         </is>
       </c>
       <c r="BF41" t="inlineStr">
         <is>
-          <t>EYE</t>
+          <t>GAS</t>
         </is>
       </c>
       <c r="BG41" t="inlineStr">
         <is>
-          <t>eyewash</t>
+          <t>gas cylinder</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>workspace</t>
+          <t>window</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>working area that must stay clear</t>
+          <t>mount = wall, z = sill height</t>
         </is>
       </c>
       <c r="BF42" t="inlineStr">
         <is>
-          <t>COL</t>
+          <t>EYE</t>
         </is>
       </c>
       <c r="BG42" t="inlineStr">
         <is>
-          <t>column</t>
+          <t>eyewash</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>overhead</t>
+          <t>workspace</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>duct, beam, cable tray, light: mount = wall, z = underside</t>
+          <t>working area that must stay clear</t>
         </is>
       </c>
       <c r="BF43" t="inlineStr">
         <is>
-          <t>PANEL</t>
+          <t>COL</t>
         </is>
       </c>
       <c r="BG43" t="inlineStr">
         <is>
-          <t>electrical panel</t>
+          <t>column</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t>overhead</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>duct, beam, cable tray, light: mount = wall, z = underside</t>
+        </is>
+      </c>
+      <c r="BF44" t="inlineStr">
+        <is>
+          <t>PANEL</t>
+        </is>
+      </c>
+      <c r="BG44" t="inlineStr">
+        <is>
+          <t>electrical panel</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t>other</t>
         </is>
       </c>
-      <c r="BF44" t="inlineStr">
+      <c r="BF45" t="inlineStr">
         <is>
           <t>DOOR</t>
         </is>
       </c>
-      <c r="BG44" t="inlineStr">
+      <c r="BG45" t="inlineStr">
         <is>
           <t>door</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="BF45" t="inlineStr">
-        <is>
-          <t>WIN</t>
-        </is>
-      </c>
-      <c r="BG45" t="inlineStr">
-        <is>
-          <t>window</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="BF46" t="inlineStr">
         <is>
-          <t>WS</t>
+          <t>WIN</t>
         </is>
       </c>
       <c r="BG46" t="inlineStr">
         <is>
-          <t>workspace</t>
+          <t>window</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="BF47" t="inlineStr">
         <is>
-          <t>DUCT</t>
+          <t>WS</t>
         </is>
       </c>
       <c r="BG47" t="inlineStr">
         <is>
-          <t>duct / overhead</t>
+          <t>workspace</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="BF48" t="inlineStr">
         <is>
-          <t>OUT</t>
+          <t>DUCT</t>
         </is>
       </c>
       <c r="BG48" t="inlineStr">
         <is>
-          <t>outlet</t>
+          <t>duct / overhead</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="BF49" t="inlineStr">
         <is>
-          <t>STRIP</t>
+          <t>OUT</t>
         </is>
       </c>
       <c r="BG49" t="inlineStr">
         <is>
-          <t>power strip</t>
+          <t>outlet</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="BF50" t="inlineStr">
         <is>
-          <t>NET</t>
+          <t>STRIP</t>
         </is>
       </c>
       <c r="BG50" t="inlineStr">
         <is>
-          <t>network port</t>
+          <t>power strip</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="BF51" t="inlineStr">
         <is>
-          <t>GASTAP</t>
+          <t>NET</t>
         </is>
       </c>
       <c r="BG51" t="inlineStr">
         <is>
-          <t>gas tap</t>
+          <t>network port</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="BF52" t="inlineStr">
         <is>
-          <t>EXH</t>
+          <t>GASTAP</t>
         </is>
       </c>
       <c r="BG52" t="inlineStr">
         <is>
-          <t>extraction point</t>
+          <t>gas tap</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="BF53" t="inlineStr">
         <is>
-          <t>EARTH</t>
+          <t>EXH</t>
         </is>
       </c>
       <c r="BG53" t="inlineStr">
         <is>
-          <t>earth point</t>
+          <t>extraction point</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="BF54" t="inlineStr">
         <is>
-          <t>X.A  X.B</t>
+          <t>EARTH</t>
         </is>
       </c>
       <c r="BG54" t="inlineStr">
         <is>
-          <t>parts of a composed object</t>
+          <t>earth point</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="BF55" t="inlineStr">
         <is>
-          <t>X.D1  X.D2</t>
+          <t>X.A  X.B</t>
         </is>
       </c>
       <c r="BG55" t="inlineStr">
         <is>
-          <t>drawers, numbered from the top</t>
+          <t>parts of a composed object</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="BF56" t="inlineStr">
         <is>
-          <t>X.S1  X.S2</t>
+          <t>X.D1  X.D2</t>
         </is>
       </c>
       <c r="BG56" t="inlineStr">
         <is>
-          <t>shelves, numbered from the top</t>
+          <t>drawers, numbered from the top</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="BF57" t="inlineStr">
         <is>
+          <t>X.S1  X.S2</t>
+        </is>
+      </c>
+      <c r="BG57" t="inlineStr">
+        <is>
+          <t>shelves, numbered from the top</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="BF58" t="inlineStr">
+        <is>
           <t>I-0001</t>
         </is>
       </c>
-      <c r="BG57" t="inlineStr">
+      <c r="BG58" t="inlineStr">
         <is>
           <t>items: just number them</t>
         </is>

</xml_diff>